<commit_message>
Updated ASR Multi Engines
</commit_message>
<xml_diff>
--- a/asr_lab_pro_logs.xlsx
+++ b/asr_lab_pro_logs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2415,6 +2415,308 @@
         <v>0</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>–phin game dance?因為伝öv.. … dumplings are doing lol –so we are not going to die anymore – Finning music please –Ok Supra ritual тепール –and just talk about how we belong Boy, I like dancing – Hello –Mrs. –Yes –Yes –ande del bowling –Very fine кто Moscow Opera Big Khóvkum? Any points. then stage. That's the every meaning sometimes. Saqabam,자�ытか klisvious negativeurna and evolve phase two and кнопal orthogonal factor attained t. Otherwise you're way too responsible. Saqabam,حats venture. Pa sorrajarya,eud zenhan Ramadan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>46.881</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1.0244</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:25:30</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>45.767</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="P32" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+      <c r="R32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Faster-Whisper</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>– K physicalią gallons, – Kr visualization – Ar medication or poo seems to be American medicine now. – Kr visualization – Kr thinking how to perform Roman medicine? – Kr thinking how to perform Sri Kerala – Kr thinking about freed nectar of我 – Kr thinking about favourful and divine meditation? – Kr thought, what a third person can say is that – Kr thinking about Ihrer.. – Kr thinking about cheating him but neither逛ligations! – Kr thinking about abhairs and knowing himself, – Kr thinking about百.. Nobody is talking about that. So, I will take care of that. Yes, you have got a lot of trouble. What I can get a glass of water. Yes, I will get it.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>21.243</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.4642</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.1641</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:25:30</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>45.767</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="P33" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Faster-Whisper</t>
+        </is>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sarvam AI</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Audio 45.8s &gt; 30s limit</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:25:30</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>45.767</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="P34" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Sarvam AI</t>
+        </is>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>IndicConformer</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>You are trying to access a gated repo.
+Make sure to have access to it at https://huggingface.co/ai4bharat/indic-conformer-600m-multilingual.
+403 Client Error. (Request ID: Root=1-6a4c94cf-6403e5e65a27</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:25:30</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>45.767</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="P35" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>IndicConformer</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>IndicWav2Vec</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>You are trying to access a gated repo.
+Make sure to have access to it at https://huggingface.co/ai4bharat/indicwav2vec_v1_hindi.
+403 Client Error. (Request ID: Root=1-6a4c94d0-7a40fef01e428c6039e62eff</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-07-07T11:25:30</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>45.767</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>🌐 Auto Detect</t>
+        </is>
+      </c>
+      <c r="P36" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>IndicWav2Vec</t>
+        </is>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>